<commit_message>
add module 3 and 4
</commit_message>
<xml_diff>
--- a/backend/ventas_reporte.xlsx
+++ b/backend/ventas_reporte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1094,6 +1094,27 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1144.65</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-04-14 03:10:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>